<commit_message>
fix - fillable model
</commit_message>
<xml_diff>
--- a/public/format_file_excel_import/struktur_umur_penduduk_status_kawin_kelompok_umur.xlsx
+++ b/public/format_file_excel_import/struktur_umur_penduduk_status_kawin_kelompok_umur.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ariesyarwani/Documents/format excel import/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\my_project\rumah_data\public\format_file_excel_import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40FCABF8-243A-EF4F-AFEB-76B393C541CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3296F400-A18B-4EF7-A604-C08B08772B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1240" windowWidth="27640" windowHeight="16760" xr2:uid="{8BDDEE65-8005-AC46-A92E-A8CDF641EE4D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8BDDEE65-8005-AC46-A92E-A8CDF641EE4D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -287,9 +287,6 @@
     <t>50_54_belum_kawin_pr</t>
   </si>
   <si>
-    <t>50_54_kawin _lk</t>
-  </si>
-  <si>
     <t>50_54_kawin_pr</t>
   </si>
   <si>
@@ -423,6 +420,9 @@
   </si>
   <si>
     <t>lebih_75_cerai_mati_pr</t>
+  </si>
+  <si>
+    <t>50_54_kawin_lk</t>
   </si>
 </sst>
 </file>
@@ -590,7 +590,7 @@
     <tableColumn id="81" xr3:uid="{3906D31B-2D37-704D-A2FA-3A4D3800E987}" name="45_49_cerai_mati_pr"/>
     <tableColumn id="82" xr3:uid="{ECCA9591-E297-3646-8B5B-15DDC312E4B1}" name="50_54_belum_kawin_lk"/>
     <tableColumn id="83" xr3:uid="{D416C3B0-BE41-0649-8101-C7C39DFAAE40}" name="50_54_belum_kawin_pr"/>
-    <tableColumn id="84" xr3:uid="{05E09139-185C-F948-9452-274C4D37473F}" name="50_54_kawin _lk"/>
+    <tableColumn id="84" xr3:uid="{05E09139-185C-F948-9452-274C4D37473F}" name="50_54_kawin_lk"/>
     <tableColumn id="85" xr3:uid="{AFAE5EA0-BE0D-E44F-BDD8-9BEF148EBD39}" name="50_54_kawin_pr"/>
     <tableColumn id="86" xr3:uid="{55B6A811-9304-394F-A369-5CA3001AE046}" name="50_54_cerai_hidup_lk"/>
     <tableColumn id="87" xr3:uid="{932F5C98-86FD-7B4F-A141-D55161CE8731}" name="50_54_cerai_hidup_pr"/>
@@ -959,140 +959,140 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8965B77-8B2A-3D4D-9CF5-1DAC9C42C87F}">
   <dimension ref="A1:DY129"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="22.375" customWidth="1"/>
     <col min="3" max="3" width="22.5" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.375" customWidth="1"/>
     <col min="5" max="5" width="16.5" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
-    <col min="7" max="7" width="21.1640625" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="21.125" customWidth="1"/>
+    <col min="8" max="8" width="20.375" customWidth="1"/>
     <col min="9" max="9" width="20.5" customWidth="1"/>
-    <col min="10" max="10" width="22.33203125" customWidth="1"/>
+    <col min="10" max="10" width="22.375" customWidth="1"/>
     <col min="11" max="11" width="22.5" customWidth="1"/>
-    <col min="12" max="12" width="16.33203125" customWidth="1"/>
+    <col min="12" max="12" width="16.375" customWidth="1"/>
     <col min="13" max="13" width="16.5" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="21.1640625" customWidth="1"/>
-    <col min="16" max="16" width="20.33203125" customWidth="1"/>
+    <col min="15" max="15" width="21.125" customWidth="1"/>
+    <col min="16" max="16" width="20.375" customWidth="1"/>
     <col min="17" max="17" width="20.5" customWidth="1"/>
-    <col min="18" max="18" width="22.33203125" customWidth="1"/>
+    <col min="18" max="18" width="22.375" customWidth="1"/>
     <col min="19" max="19" width="22.5" customWidth="1"/>
-    <col min="20" max="20" width="16.33203125" customWidth="1"/>
+    <col min="20" max="20" width="16.375" customWidth="1"/>
     <col min="21" max="21" width="16.5" customWidth="1"/>
     <col min="22" max="22" width="21" customWidth="1"/>
-    <col min="23" max="23" width="21.1640625" customWidth="1"/>
-    <col min="24" max="24" width="20.33203125" customWidth="1"/>
+    <col min="23" max="23" width="21.125" customWidth="1"/>
+    <col min="24" max="24" width="20.375" customWidth="1"/>
     <col min="25" max="25" width="20.5" customWidth="1"/>
-    <col min="26" max="26" width="22.33203125" customWidth="1"/>
+    <col min="26" max="26" width="22.375" customWidth="1"/>
     <col min="27" max="27" width="22.5" customWidth="1"/>
-    <col min="28" max="28" width="16.33203125" customWidth="1"/>
+    <col min="28" max="28" width="16.375" customWidth="1"/>
     <col min="29" max="29" width="16.5" customWidth="1"/>
     <col min="30" max="30" width="21" customWidth="1"/>
-    <col min="31" max="31" width="21.1640625" customWidth="1"/>
-    <col min="32" max="32" width="20.33203125" customWidth="1"/>
+    <col min="31" max="31" width="21.125" customWidth="1"/>
+    <col min="32" max="32" width="20.375" customWidth="1"/>
     <col min="33" max="33" width="20.5" customWidth="1"/>
-    <col min="34" max="34" width="22.33203125" customWidth="1"/>
+    <col min="34" max="34" width="22.375" customWidth="1"/>
     <col min="35" max="35" width="22.5" customWidth="1"/>
-    <col min="36" max="36" width="16.33203125" customWidth="1"/>
+    <col min="36" max="36" width="16.375" customWidth="1"/>
     <col min="37" max="37" width="16.5" customWidth="1"/>
     <col min="38" max="38" width="21" customWidth="1"/>
-    <col min="39" max="39" width="21.1640625" customWidth="1"/>
-    <col min="40" max="40" width="20.33203125" customWidth="1"/>
+    <col min="39" max="39" width="21.125" customWidth="1"/>
+    <col min="40" max="40" width="20.375" customWidth="1"/>
     <col min="41" max="41" width="20.5" customWidth="1"/>
-    <col min="42" max="42" width="22.33203125" customWidth="1"/>
+    <col min="42" max="42" width="22.375" customWidth="1"/>
     <col min="43" max="43" width="22.5" customWidth="1"/>
-    <col min="44" max="44" width="16.33203125" customWidth="1"/>
+    <col min="44" max="44" width="16.375" customWidth="1"/>
     <col min="45" max="45" width="16.5" customWidth="1"/>
     <col min="46" max="46" width="21" customWidth="1"/>
-    <col min="47" max="47" width="21.1640625" customWidth="1"/>
-    <col min="48" max="48" width="20.33203125" customWidth="1"/>
+    <col min="47" max="47" width="21.125" customWidth="1"/>
+    <col min="48" max="48" width="20.375" customWidth="1"/>
     <col min="49" max="49" width="20.5" customWidth="1"/>
-    <col min="50" max="50" width="22.33203125" customWidth="1"/>
+    <col min="50" max="50" width="22.375" customWidth="1"/>
     <col min="51" max="51" width="22.5" customWidth="1"/>
-    <col min="52" max="52" width="16.33203125" customWidth="1"/>
+    <col min="52" max="52" width="16.375" customWidth="1"/>
     <col min="53" max="53" width="16.5" customWidth="1"/>
     <col min="54" max="54" width="21" customWidth="1"/>
-    <col min="55" max="55" width="21.1640625" customWidth="1"/>
-    <col min="56" max="56" width="20.33203125" customWidth="1"/>
+    <col min="55" max="55" width="21.125" customWidth="1"/>
+    <col min="56" max="56" width="20.375" customWidth="1"/>
     <col min="57" max="57" width="20.5" customWidth="1"/>
-    <col min="58" max="58" width="22.33203125" customWidth="1"/>
+    <col min="58" max="58" width="22.375" customWidth="1"/>
     <col min="59" max="59" width="22.5" customWidth="1"/>
-    <col min="60" max="60" width="16.33203125" customWidth="1"/>
+    <col min="60" max="60" width="16.375" customWidth="1"/>
     <col min="61" max="61" width="16.5" customWidth="1"/>
     <col min="62" max="62" width="21" customWidth="1"/>
-    <col min="63" max="63" width="21.1640625" customWidth="1"/>
-    <col min="64" max="64" width="20.33203125" customWidth="1"/>
+    <col min="63" max="63" width="21.125" customWidth="1"/>
+    <col min="64" max="64" width="20.375" customWidth="1"/>
     <col min="65" max="65" width="20.5" customWidth="1"/>
-    <col min="66" max="66" width="22.33203125" customWidth="1"/>
+    <col min="66" max="66" width="22.375" customWidth="1"/>
     <col min="67" max="67" width="22.5" customWidth="1"/>
-    <col min="68" max="68" width="16.33203125" customWidth="1"/>
+    <col min="68" max="68" width="16.375" customWidth="1"/>
     <col min="69" max="69" width="16.5" customWidth="1"/>
     <col min="70" max="70" width="21" customWidth="1"/>
-    <col min="71" max="71" width="21.1640625" customWidth="1"/>
-    <col min="72" max="72" width="20.33203125" customWidth="1"/>
+    <col min="71" max="71" width="21.125" customWidth="1"/>
+    <col min="72" max="72" width="20.375" customWidth="1"/>
     <col min="73" max="73" width="20.5" customWidth="1"/>
-    <col min="74" max="74" width="22.33203125" customWidth="1"/>
+    <col min="74" max="74" width="22.375" customWidth="1"/>
     <col min="75" max="75" width="22.5" customWidth="1"/>
-    <col min="76" max="76" width="16.33203125" customWidth="1"/>
+    <col min="76" max="76" width="16.375" customWidth="1"/>
     <col min="77" max="77" width="16.5" customWidth="1"/>
     <col min="78" max="78" width="21" customWidth="1"/>
-    <col min="79" max="79" width="21.1640625" customWidth="1"/>
-    <col min="80" max="80" width="20.33203125" customWidth="1"/>
+    <col min="79" max="79" width="21.125" customWidth="1"/>
+    <col min="80" max="80" width="20.375" customWidth="1"/>
     <col min="81" max="81" width="20.5" customWidth="1"/>
-    <col min="82" max="82" width="22.33203125" customWidth="1"/>
+    <col min="82" max="82" width="22.375" customWidth="1"/>
     <col min="83" max="83" width="22.5" customWidth="1"/>
-    <col min="84" max="84" width="16.6640625" customWidth="1"/>
+    <col min="84" max="84" width="16.625" customWidth="1"/>
     <col min="85" max="85" width="16.5" customWidth="1"/>
     <col min="86" max="86" width="21" customWidth="1"/>
-    <col min="87" max="87" width="21.1640625" customWidth="1"/>
-    <col min="88" max="88" width="20.33203125" customWidth="1"/>
+    <col min="87" max="87" width="21.125" customWidth="1"/>
+    <col min="88" max="88" width="20.375" customWidth="1"/>
     <col min="89" max="89" width="20.5" customWidth="1"/>
-    <col min="90" max="90" width="22.33203125" customWidth="1"/>
+    <col min="90" max="90" width="22.375" customWidth="1"/>
     <col min="91" max="91" width="22.5" customWidth="1"/>
-    <col min="92" max="92" width="16.33203125" customWidth="1"/>
+    <col min="92" max="92" width="16.375" customWidth="1"/>
     <col min="93" max="93" width="16.5" customWidth="1"/>
     <col min="94" max="94" width="21" customWidth="1"/>
-    <col min="95" max="95" width="21.1640625" customWidth="1"/>
-    <col min="96" max="96" width="20.33203125" customWidth="1"/>
+    <col min="95" max="95" width="21.125" customWidth="1"/>
+    <col min="96" max="96" width="20.375" customWidth="1"/>
     <col min="97" max="97" width="20.5" customWidth="1"/>
-    <col min="98" max="98" width="22.33203125" customWidth="1"/>
+    <col min="98" max="98" width="22.375" customWidth="1"/>
     <col min="99" max="99" width="22.5" customWidth="1"/>
-    <col min="100" max="100" width="16.33203125" customWidth="1"/>
+    <col min="100" max="100" width="16.375" customWidth="1"/>
     <col min="101" max="101" width="16.5" customWidth="1"/>
     <col min="102" max="102" width="21" customWidth="1"/>
-    <col min="103" max="103" width="21.1640625" customWidth="1"/>
-    <col min="104" max="104" width="20.33203125" customWidth="1"/>
+    <col min="103" max="103" width="21.125" customWidth="1"/>
+    <col min="104" max="104" width="20.375" customWidth="1"/>
     <col min="105" max="105" width="20.5" customWidth="1"/>
-    <col min="106" max="106" width="22.33203125" customWidth="1"/>
+    <col min="106" max="106" width="22.375" customWidth="1"/>
     <col min="107" max="107" width="22.5" customWidth="1"/>
-    <col min="108" max="108" width="16.33203125" customWidth="1"/>
+    <col min="108" max="108" width="16.375" customWidth="1"/>
     <col min="109" max="109" width="16.5" customWidth="1"/>
     <col min="110" max="110" width="21" customWidth="1"/>
-    <col min="111" max="111" width="21.1640625" customWidth="1"/>
-    <col min="112" max="112" width="20.33203125" customWidth="1"/>
+    <col min="111" max="111" width="21.125" customWidth="1"/>
+    <col min="112" max="112" width="20.375" customWidth="1"/>
     <col min="113" max="113" width="20.5" customWidth="1"/>
-    <col min="114" max="114" width="22.33203125" customWidth="1"/>
+    <col min="114" max="114" width="22.375" customWidth="1"/>
     <col min="115" max="115" width="22.5" customWidth="1"/>
-    <col min="116" max="116" width="16.33203125" customWidth="1"/>
+    <col min="116" max="116" width="16.375" customWidth="1"/>
     <col min="117" max="117" width="16.5" customWidth="1"/>
     <col min="118" max="118" width="21" customWidth="1"/>
-    <col min="119" max="119" width="21.1640625" customWidth="1"/>
-    <col min="120" max="120" width="20.33203125" customWidth="1"/>
+    <col min="119" max="119" width="21.125" customWidth="1"/>
+    <col min="120" max="120" width="20.375" customWidth="1"/>
     <col min="121" max="121" width="20.5" customWidth="1"/>
-    <col min="122" max="122" width="24.33203125" customWidth="1"/>
+    <col min="122" max="122" width="24.375" customWidth="1"/>
     <col min="123" max="123" width="24.5" customWidth="1"/>
-    <col min="124" max="124" width="18.33203125" customWidth="1"/>
+    <col min="124" max="124" width="18.375" customWidth="1"/>
     <col min="125" max="125" width="18.5" customWidth="1"/>
     <col min="126" max="126" width="23" customWidth="1"/>
-    <col min="127" max="127" width="23.1640625" customWidth="1"/>
-    <col min="128" max="128" width="22.33203125" customWidth="1"/>
+    <col min="127" max="127" width="23.125" customWidth="1"/>
+    <col min="128" max="128" width="22.375" customWidth="1"/>
     <col min="129" max="129" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1343,526 +1343,526 @@
         <v>82</v>
       </c>
       <c r="CF1" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG1" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CH1" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CI1" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CJ1" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CK1" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CL1" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CM1" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CN1" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CO1" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CP1" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CQ1" t="s">
         <v>93</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CR1" t="s">
         <v>94</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CS1" t="s">
         <v>95</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CT1" t="s">
         <v>96</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CU1" t="s">
         <v>97</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CV1" t="s">
         <v>98</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="CW1" t="s">
         <v>99</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="CX1" t="s">
         <v>100</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="CY1" t="s">
         <v>101</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="CZ1" t="s">
         <v>102</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DA1" t="s">
         <v>103</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DB1" t="s">
         <v>104</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DC1" t="s">
         <v>105</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DD1" t="s">
         <v>106</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DE1" t="s">
         <v>107</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DF1" t="s">
         <v>108</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DG1" t="s">
         <v>109</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DH1" t="s">
         <v>110</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DI1" t="s">
         <v>111</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DJ1" t="s">
         <v>112</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DK1" t="s">
         <v>113</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DL1" t="s">
         <v>114</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DM1" t="s">
         <v>115</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DN1" t="s">
         <v>116</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DO1" t="s">
         <v>117</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DP1" t="s">
         <v>118</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DQ1" t="s">
         <v>119</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DR1" t="s">
         <v>120</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DS1" t="s">
         <v>121</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="DT1" t="s">
         <v>122</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="DU1" t="s">
         <v>123</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="DV1" t="s">
         <v>124</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="DW1" t="s">
         <v>125</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="DX1" t="s">
         <v>126</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="DY1" t="s">
         <v>127</v>
       </c>
-      <c r="DY1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="1:129" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
     </row>
-    <row r="14" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:129" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="1"/>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="1"/>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="1"/>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="1"/>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="1"/>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="1"/>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="1"/>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="1"/>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="1"/>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="1"/>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="1"/>
     </row>
   </sheetData>

</xml_diff>